<commit_message>
Lam test case 13-18
</commit_message>
<xml_diff>
--- a/Extra/TestCase_CaroGame.xlsx
+++ b/Extra/TestCase_CaroGame.xlsx
@@ -1,25 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\Network_Programming-UDM17_Group2\Extra\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Acer\Pictures\Network_Programming-UDM17_Group2\Extra\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2386D2D7-9937-43BC-A82F-0FAFC2D643AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12210"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="TC_1 Proof" sheetId="2" r:id="rId2"/>
-    <sheet name="TC_2 Proof" sheetId="3" r:id="rId3"/>
-    <sheet name="TC_3 Proof" sheetId="4" r:id="rId4"/>
-    <sheet name="TC_4 Proof" sheetId="5" r:id="rId5"/>
-    <sheet name="TC_5 Proof" sheetId="6" r:id="rId6"/>
-    <sheet name="TC_6 Proof" sheetId="7" r:id="rId7"/>
-    <sheet name="TC_7 Proof" sheetId="8" r:id="rId8"/>
+    <sheet name="TC_18 Proof" sheetId="14" r:id="rId2"/>
+    <sheet name="TC_17 Proof" sheetId="13" r:id="rId3"/>
+    <sheet name="TC_16 Proof" sheetId="12" r:id="rId4"/>
+    <sheet name="TC_15 Proof" sheetId="11" r:id="rId5"/>
+    <sheet name="TC_14 Proof" sheetId="10" r:id="rId6"/>
+    <sheet name="TC_13 Proof" sheetId="9" r:id="rId7"/>
+    <sheet name="TC_1 Proof" sheetId="2" r:id="rId8"/>
+    <sheet name="TC_2 Proof" sheetId="3" r:id="rId9"/>
+    <sheet name="TC_3 Proof" sheetId="4" r:id="rId10"/>
+    <sheet name="TC_4 Proof" sheetId="5" r:id="rId11"/>
+    <sheet name="TC_5 Proof" sheetId="6" r:id="rId12"/>
+    <sheet name="TC_6 Proof" sheetId="7" r:id="rId13"/>
+    <sheet name="TC_7 Proof" sheetId="8" r:id="rId14"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -31,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="171">
   <si>
     <t>No</t>
   </si>
@@ -534,16 +541,37 @@
   <si>
     <t>Server xử lý disconnect đúng quy trình, tin nhắn đã gửi trước đó không bị mất ở phía người nhận (nếu đã đến server)</t>
   </si>
+  <si>
+    <t>TC_13 Proof</t>
+  </si>
+  <si>
+    <t>TC_14 Proof</t>
+  </si>
+  <si>
+    <t>TC_15 Proof</t>
+  </si>
+  <si>
+    <t>TC_16 Proof</t>
+  </si>
+  <si>
+    <t>TC_17 Proof</t>
+  </si>
+  <si>
+    <t>TC_18 Proof</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="163"/>
       <scheme val="minor"/>
@@ -588,7 +616,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -613,15 +641,23 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>266700</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>477337</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>29377</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1"/>
-        <xdr:cNvPicPr/>
+        <xdr:cNvPr id="3" name="Hình ảnh 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{783469DE-B3E5-E019-6078-CF6D9253754E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
@@ -632,7 +668,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="7124700" cy="4191000"/>
+          <a:ext cx="7792537" cy="5744377"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -644,89 +680,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>409574</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>66675</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="7953374" cy="4772025"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>314324</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>161925</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="9915524" cy="5772150"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -743,7 +697,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -767,7 +727,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -784,7 +744,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -810,7 +776,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -827,7 +793,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -853,7 +825,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -870,7 +842,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -885,6 +863,392 @@
         <a:xfrm>
           <a:off x="0" y="0"/>
           <a:ext cx="10571428" cy="7142857"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>534495</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>124587</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Hình ảnh 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F4731257-A2F5-E0C0-4098-21CE5D7269E5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7849695" cy="5458587"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>334868</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>124826</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Hình ảnh 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1284504C-390E-EFF4-4A7D-05221E2B66B2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="10698068" cy="7173326"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>353921</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>96247</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Hình ảnh 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ADBE2B7C-70F3-C736-F1A8-90B674263D2E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="10717121" cy="7144747"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>601180</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>172192</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Hình ảnh 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7220D5AD-0D92-889B-636A-187BD8B1F98E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7916380" cy="5315692"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>553548</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>162665</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Hình ảnh 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AE1E81C6-E475-60A2-FA31-9E666D63DEBE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7868748" cy="5306165"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>266700</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7124700" cy="4191000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>409574</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7953374" cy="4772025"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>314324</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="9915524" cy="5772150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1158,16 +1522,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:H32"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="9" customWidth="1"/>
-    <col min="3" max="3" width="32.625" customWidth="1"/>
-    <col min="4" max="4" width="28.875" customWidth="1"/>
-    <col min="5" max="5" width="55.25" customWidth="1"/>
-    <col min="6" max="6" width="72.5" customWidth="1"/>
-    <col min="7" max="7" width="15.625" customWidth="1"/>
+    <col min="3" max="3" width="32.5703125" customWidth="1"/>
+    <col min="4" max="4" width="28.85546875" customWidth="1"/>
+    <col min="5" max="5" width="55.28515625" customWidth="1"/>
+    <col min="6" max="6" width="72.42578125" customWidth="1"/>
+    <col min="7" max="7" width="15.5703125" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1456,6 +1820,12 @@
       <c r="F15" s="2" t="s">
         <v>78</v>
       </c>
+      <c r="G15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="16" spans="2:8" ht="30" customHeight="1">
       <c r="B16" s="2" t="s">
@@ -1473,8 +1843,14 @@
       <c r="F16" s="2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="17" spans="2:6" ht="30" customHeight="1">
+      <c r="G16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" ht="30" customHeight="1">
       <c r="B17" s="2" t="s">
         <v>84</v>
       </c>
@@ -1490,8 +1866,14 @@
       <c r="F17" s="2" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="18" spans="2:6" ht="45.75" customHeight="1">
+      <c r="G17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" ht="45.75" customHeight="1">
       <c r="B18" s="2" t="s">
         <v>89</v>
       </c>
@@ -1507,8 +1889,14 @@
       <c r="F18" s="2" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="19" spans="2:6" ht="27" customHeight="1">
+      <c r="G18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" ht="27" customHeight="1">
       <c r="B19" s="2" t="s">
         <v>94</v>
       </c>
@@ -1524,8 +1912,14 @@
       <c r="F19" s="2" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="20" spans="2:6" ht="45" customHeight="1">
+      <c r="G19" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" ht="45" customHeight="1">
       <c r="B20" s="2" t="s">
         <v>99</v>
       </c>
@@ -1541,8 +1935,14 @@
       <c r="F20" s="2" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="21" spans="2:6" ht="27.75" customHeight="1">
+      <c r="G20" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" ht="27.75" customHeight="1">
       <c r="B21" t="s">
         <v>104</v>
       </c>
@@ -1559,7 +1959,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="22" spans="2:6" ht="45.75" customHeight="1">
+    <row r="22" spans="2:8" ht="45.75" customHeight="1">
       <c r="B22" t="s">
         <v>109</v>
       </c>
@@ -1576,7 +1976,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="23" spans="2:6" ht="36" customHeight="1">
+    <row r="23" spans="2:8" ht="36" customHeight="1">
       <c r="B23" t="s">
         <v>114</v>
       </c>
@@ -1593,7 +1993,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="24" spans="2:6" ht="27" customHeight="1">
+    <row r="24" spans="2:8" ht="27" customHeight="1">
       <c r="B24" s="2" t="s">
         <v>119</v>
       </c>
@@ -1610,7 +2010,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="25" spans="2:6" ht="30.75" customHeight="1">
+    <row r="25" spans="2:8" ht="30.75" customHeight="1">
       <c r="B25" s="2" t="s">
         <v>124</v>
       </c>
@@ -1627,7 +2027,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="26" spans="2:6" ht="28.5">
+    <row r="26" spans="2:8" ht="30">
       <c r="B26" s="2" t="s">
         <v>129</v>
       </c>
@@ -1644,7 +2044,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="27" spans="2:6" ht="18.75" customHeight="1">
+    <row r="27" spans="2:8" ht="18.75" customHeight="1">
       <c r="B27" s="2" t="s">
         <v>134</v>
       </c>
@@ -1661,7 +2061,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="28" spans="2:6" ht="28.5" customHeight="1">
+    <row r="28" spans="2:8" ht="28.5" customHeight="1">
       <c r="B28" s="2" t="s">
         <v>139</v>
       </c>
@@ -1678,7 +2078,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="29" spans="2:6" ht="28.5">
+    <row r="29" spans="2:8" ht="30">
       <c r="B29" s="2" t="s">
         <v>144</v>
       </c>
@@ -1695,7 +2095,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="30" spans="2:6" ht="28.5">
+    <row r="30" spans="2:8" ht="30">
       <c r="B30" s="2" t="s">
         <v>149</v>
       </c>
@@ -1712,7 +2112,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="31" spans="2:6" ht="28.5">
+    <row r="31" spans="2:8" ht="30">
       <c r="B31" s="2" t="s">
         <v>154</v>
       </c>
@@ -1729,7 +2129,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="32" spans="2:6" ht="28.5">
+    <row r="32" spans="2:8" ht="30">
       <c r="B32" s="2" t="s">
         <v>159</v>
       </c>
@@ -1751,70 +2151,130 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76C502C3-D955-4D43-92AC-197D467819DA}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53934063-2735-4DD6-AE8A-2E07110B0DE2}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA8E1100-81A7-4F1E-9E74-9C0D79583CC0}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2BB8AA3-EE47-42D9-9FD1-F60BB28F77BC}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F556CF5-6313-4FF1-92FA-DCCD167DC3F3}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{687273F0-2DA0-4B20-9854-E83AD0907408}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>